<commit_message>
Actualizar buscador de placas
</commit_message>
<xml_diff>
--- a/consultas/conductor.xlsx
+++ b/consultas/conductor.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showInkAnnotation="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jefferson\Desktop\consultas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jefferson\Desktop\ATU\atu app\consultas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{680FC098-311E-4E49-A80C-129EF9BFC795}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{917730F5-853C-473E-94AE-B691660B4D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="509">
   <si>
     <t>CARRILLO PITO RONY OSWALDO</t>
   </si>
@@ -1985,7 +1985,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{179EC4C1-829A-F14A-B4CA-A933AB5EC71A}">
-  <dimension ref="A1:D329"/>
+  <dimension ref="A1:E329"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="35.33203125" customWidth="1"/>
@@ -4456,7 +4456,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>426057</v>
       </c>
@@ -4470,7 +4470,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>426496</v>
       </c>
@@ -4484,7 +4484,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>425760</v>
       </c>
@@ -4498,7 +4498,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>426646</v>
       </c>
@@ -4512,7 +4512,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>426409</v>
       </c>
@@ -4522,8 +4522,14 @@
       <c r="C181">
         <v>9765665</v>
       </c>
-    </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D181" t="s">
+        <v>423</v>
+      </c>
+      <c r="E181">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>426329</v>
       </c>
@@ -4533,8 +4539,14 @@
       <c r="C182">
         <v>45780665</v>
       </c>
-    </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D182" t="s">
+        <v>424</v>
+      </c>
+      <c r="E182">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>426599</v>
       </c>
@@ -4544,8 +4556,14 @@
       <c r="C183">
         <v>44030322</v>
       </c>
-    </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D183" t="s">
+        <v>425</v>
+      </c>
+      <c r="E183">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>425253</v>
       </c>
@@ -4555,8 +4573,14 @@
       <c r="C184">
         <v>41029743</v>
       </c>
-    </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D184" t="s">
+        <v>426</v>
+      </c>
+      <c r="E184">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>425314</v>
       </c>
@@ -4566,8 +4590,14 @@
       <c r="C185">
         <v>40994351</v>
       </c>
-    </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D185" t="s">
+        <v>417</v>
+      </c>
+      <c r="E185">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>426491</v>
       </c>
@@ -4577,8 +4607,14 @@
       <c r="C186">
         <v>45861364</v>
       </c>
-    </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D186" t="s">
+        <v>418</v>
+      </c>
+      <c r="E186">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>426394</v>
       </c>
@@ -4588,8 +4624,14 @@
       <c r="C187">
         <v>9736732</v>
       </c>
-    </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D187" t="s">
+        <v>419</v>
+      </c>
+      <c r="E187">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>425163</v>
       </c>
@@ -4599,8 +4641,14 @@
       <c r="C188">
         <v>43521051</v>
       </c>
-    </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D188" t="s">
+        <v>416</v>
+      </c>
+      <c r="E188">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>425271</v>
       </c>
@@ -4610,8 +4658,14 @@
       <c r="C189">
         <v>46314815</v>
       </c>
-    </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D189" t="s">
+        <v>427</v>
+      </c>
+      <c r="E189">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>426370</v>
       </c>
@@ -4621,8 +4675,14 @@
       <c r="C190">
         <v>10240845</v>
       </c>
-    </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D190" t="s">
+        <v>386</v>
+      </c>
+      <c r="E190">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>425254</v>
       </c>
@@ -4632,8 +4692,14 @@
       <c r="C191">
         <v>9987483</v>
       </c>
-    </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D191" t="s">
+        <v>393</v>
+      </c>
+      <c r="E191">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>426064</v>
       </c>
@@ -4643,8 +4709,14 @@
       <c r="C192">
         <v>46714230</v>
       </c>
-    </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D192" t="s">
+        <v>396</v>
+      </c>
+      <c r="E192">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>425479</v>
       </c>
@@ -4654,8 +4726,14 @@
       <c r="C193">
         <v>9548620</v>
       </c>
-    </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D193" t="s">
+        <v>395</v>
+      </c>
+      <c r="E193">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>425282</v>
       </c>
@@ -4665,8 +4743,14 @@
       <c r="C194">
         <v>10112492</v>
       </c>
-    </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D194" t="s">
+        <v>398</v>
+      </c>
+      <c r="E194">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>425713</v>
       </c>
@@ -4676,8 +4760,14 @@
       <c r="C195">
         <v>43691346</v>
       </c>
-    </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D195" t="s">
+        <v>397</v>
+      </c>
+      <c r="E195">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>425305</v>
       </c>
@@ -4687,8 +4777,14 @@
       <c r="C196">
         <v>23714604</v>
       </c>
-    </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D196" t="s">
+        <v>399</v>
+      </c>
+      <c r="E196">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>426304</v>
       </c>
@@ -4698,8 +4794,14 @@
       <c r="C197">
         <v>46666538</v>
       </c>
-    </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D197" t="s">
+        <v>394</v>
+      </c>
+      <c r="E197">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>425383</v>
       </c>
@@ -4709,8 +4811,14 @@
       <c r="C198">
         <v>47061654</v>
       </c>
-    </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D198" t="s">
+        <v>429</v>
+      </c>
+      <c r="E198">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>425377</v>
       </c>
@@ -4720,8 +4828,14 @@
       <c r="C199">
         <v>9097433</v>
       </c>
-    </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D199" t="s">
+        <v>430</v>
+      </c>
+      <c r="E199">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>425356</v>
       </c>
@@ -4731,8 +4845,14 @@
       <c r="C200">
         <v>10108715</v>
       </c>
-    </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D200" t="s">
+        <v>431</v>
+      </c>
+      <c r="E200">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>426251</v>
       </c>
@@ -4742,8 +4862,14 @@
       <c r="C201">
         <v>461255</v>
       </c>
-    </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D201" t="s">
+        <v>432</v>
+      </c>
+      <c r="E201">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>425931</v>
       </c>
@@ -4753,8 +4879,14 @@
       <c r="C202">
         <v>46224702</v>
       </c>
-    </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D202" t="s">
+        <v>433</v>
+      </c>
+      <c r="E202">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>426731</v>
       </c>
@@ -4764,8 +4896,14 @@
       <c r="C203">
         <v>41521058</v>
       </c>
-    </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D203" t="s">
+        <v>434</v>
+      </c>
+      <c r="E203">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>426053</v>
       </c>
@@ -4775,8 +4913,14 @@
       <c r="C204">
         <v>44378202</v>
       </c>
-    </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D204" t="s">
+        <v>435</v>
+      </c>
+      <c r="E204">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>426389</v>
       </c>
@@ -4786,8 +4930,14 @@
       <c r="C205">
         <v>43617797</v>
       </c>
-    </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D205" t="s">
+        <v>436</v>
+      </c>
+      <c r="E205">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>410000</v>
       </c>
@@ -4797,8 +4947,14 @@
       <c r="C206">
         <v>8170426</v>
       </c>
-    </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D206" t="s">
+        <v>437</v>
+      </c>
+      <c r="E206">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>426076</v>
       </c>
@@ -4808,8 +4964,14 @@
       <c r="C207">
         <v>44858581</v>
       </c>
-    </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D207" t="s">
+        <v>438</v>
+      </c>
+      <c r="E207">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>426497</v>
       </c>
@@ -4819,8 +4981,14 @@
       <c r="C208">
         <v>8335034</v>
       </c>
-    </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D208" t="s">
+        <v>439</v>
+      </c>
+      <c r="E208">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>426396</v>
       </c>
@@ -4830,8 +4998,14 @@
       <c r="C209">
         <v>42395998</v>
       </c>
-    </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D209" t="s">
+        <v>440</v>
+      </c>
+      <c r="E209">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>426627</v>
       </c>
@@ -4841,8 +5015,14 @@
       <c r="C210">
         <v>10560331</v>
       </c>
-    </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D210" t="s">
+        <v>441</v>
+      </c>
+      <c r="E210">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>426153</v>
       </c>
@@ -4852,8 +5032,14 @@
       <c r="C211">
         <v>40987140</v>
       </c>
-    </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D211" t="s">
+        <v>442</v>
+      </c>
+      <c r="E211">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>425860</v>
       </c>
@@ -4863,8 +5049,14 @@
       <c r="C212">
         <v>10516769</v>
       </c>
-    </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D212" t="s">
+        <v>443</v>
+      </c>
+      <c r="E212">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>426740</v>
       </c>
@@ -4874,8 +5066,14 @@
       <c r="C213">
         <v>10121211</v>
       </c>
-    </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D213" t="s">
+        <v>444</v>
+      </c>
+      <c r="E213">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>426638</v>
       </c>
@@ -4885,8 +5083,14 @@
       <c r="C214">
         <v>42893019</v>
       </c>
-    </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D214" t="s">
+        <v>445</v>
+      </c>
+      <c r="E214">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>425921</v>
       </c>
@@ -4896,8 +5100,14 @@
       <c r="C215">
         <v>9097719</v>
       </c>
-    </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D215" t="s">
+        <v>446</v>
+      </c>
+      <c r="E215">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>426600</v>
       </c>
@@ -4907,8 +5117,14 @@
       <c r="C216">
         <v>45201845</v>
       </c>
-    </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D216" t="s">
+        <v>447</v>
+      </c>
+      <c r="E216">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>426042</v>
       </c>
@@ -4918,8 +5134,14 @@
       <c r="C217">
         <v>40440738</v>
       </c>
-    </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D217" t="s">
+        <v>448</v>
+      </c>
+      <c r="E217">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>426471</v>
       </c>
@@ -4929,8 +5151,14 @@
       <c r="C218">
         <v>8018176</v>
       </c>
-    </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D218" t="s">
+        <v>449</v>
+      </c>
+      <c r="E218">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>426481</v>
       </c>
@@ -4940,8 +5168,14 @@
       <c r="C219">
         <v>8527398</v>
       </c>
-    </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D219" t="s">
+        <v>450</v>
+      </c>
+      <c r="E219">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>425922</v>
       </c>
@@ -4951,8 +5185,14 @@
       <c r="C220">
         <v>42627738</v>
       </c>
-    </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D220" t="s">
+        <v>451</v>
+      </c>
+      <c r="E220">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>426640</v>
       </c>
@@ -4962,8 +5202,14 @@
       <c r="C221">
         <v>43885653</v>
       </c>
-    </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D221" t="s">
+        <v>452</v>
+      </c>
+      <c r="E221">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>426732</v>
       </c>
@@ -4973,8 +5219,14 @@
       <c r="C222">
         <v>44973710</v>
       </c>
-    </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D222" t="s">
+        <v>453</v>
+      </c>
+      <c r="E222">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="223" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>426767</v>
       </c>
@@ -4984,8 +5236,14 @@
       <c r="C223">
         <v>44515825</v>
       </c>
-    </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D223" t="s">
+        <v>454</v>
+      </c>
+      <c r="E223">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>426186</v>
       </c>
@@ -4995,8 +5253,14 @@
       <c r="C224">
         <v>7535983</v>
       </c>
-    </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D224" t="s">
+        <v>455</v>
+      </c>
+      <c r="E224">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>426309</v>
       </c>
@@ -5006,8 +5270,14 @@
       <c r="C225">
         <v>42982981</v>
       </c>
-    </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D225" t="s">
+        <v>456</v>
+      </c>
+      <c r="E225">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>415633</v>
       </c>
@@ -5017,8 +5287,14 @@
       <c r="C226">
         <v>9655568</v>
       </c>
-    </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D226" t="s">
+        <v>457</v>
+      </c>
+      <c r="E226">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>426060</v>
       </c>
@@ -5028,8 +5304,14 @@
       <c r="C227">
         <v>23242736</v>
       </c>
-    </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D227" t="s">
+        <v>458</v>
+      </c>
+      <c r="E227">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>426601</v>
       </c>
@@ -5039,8 +5321,14 @@
       <c r="C228">
         <v>43572194</v>
       </c>
-    </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D228" t="s">
+        <v>459</v>
+      </c>
+      <c r="E228">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>426035</v>
       </c>
@@ -5050,8 +5338,14 @@
       <c r="C229">
         <v>20071919</v>
       </c>
-    </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D229" t="s">
+        <v>460</v>
+      </c>
+      <c r="E229">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>426004</v>
       </c>
@@ -5061,8 +5355,14 @@
       <c r="C230">
         <v>22703794</v>
       </c>
-    </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D230" t="s">
+        <v>461</v>
+      </c>
+      <c r="E230">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>426455</v>
       </c>
@@ -5072,8 +5372,14 @@
       <c r="C231">
         <v>25499826</v>
       </c>
-    </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D231" t="s">
+        <v>462</v>
+      </c>
+      <c r="E231">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="232" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>426647</v>
       </c>
@@ -5083,8 +5389,14 @@
       <c r="C232">
         <v>46763379</v>
       </c>
-    </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D232" t="s">
+        <v>463</v>
+      </c>
+      <c r="E232">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="233" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>426410</v>
       </c>
@@ -5094,8 +5406,14 @@
       <c r="C233">
         <v>41415699</v>
       </c>
-    </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D233" t="s">
+        <v>464</v>
+      </c>
+      <c r="E233">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>425727</v>
       </c>
@@ -5105,8 +5423,14 @@
       <c r="C234">
         <v>44102709</v>
       </c>
-    </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D234" t="s">
+        <v>465</v>
+      </c>
+      <c r="E234">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>426454</v>
       </c>
@@ -5116,8 +5440,14 @@
       <c r="C235">
         <v>42958617</v>
       </c>
-    </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D235" t="s">
+        <v>466</v>
+      </c>
+      <c r="E235">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="236" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>415505</v>
       </c>
@@ -5127,8 +5457,14 @@
       <c r="C236">
         <v>43715072</v>
       </c>
-    </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D236" t="s">
+        <v>467</v>
+      </c>
+      <c r="E236">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="237" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>425903</v>
       </c>
@@ -5138,8 +5474,14 @@
       <c r="C237">
         <v>961968</v>
       </c>
-    </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D237" t="s">
+        <v>470</v>
+      </c>
+      <c r="E237">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="238" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>425748</v>
       </c>
@@ -5149,8 +5491,14 @@
       <c r="C238">
         <v>40784512</v>
       </c>
-    </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D238" t="s">
+        <v>468</v>
+      </c>
+      <c r="E238">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="239" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>425793</v>
       </c>
@@ -5160,8 +5508,14 @@
       <c r="C239">
         <v>8690779</v>
       </c>
-    </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D239" t="s">
+        <v>473</v>
+      </c>
+      <c r="E239">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>425798</v>
       </c>
@@ -5171,8 +5525,14 @@
       <c r="C240">
         <v>43382751</v>
       </c>
-    </row>
-    <row r="241" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D240" t="s">
+        <v>472</v>
+      </c>
+      <c r="E240">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="241" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>426291</v>
       </c>
@@ -5182,8 +5542,14 @@
       <c r="C241">
         <v>20568099</v>
       </c>
-    </row>
-    <row r="242" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D241" t="s">
+        <v>471</v>
+      </c>
+      <c r="E241">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="242" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>426774</v>
       </c>
@@ -5193,8 +5559,14 @@
       <c r="C242">
         <v>26719317</v>
       </c>
-    </row>
-    <row r="243" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D242" t="s">
+        <v>469</v>
+      </c>
+      <c r="E242">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="243" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>415634</v>
       </c>
@@ -5204,8 +5576,14 @@
       <c r="C243">
         <v>40728414</v>
       </c>
-    </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D243" t="s">
+        <v>474</v>
+      </c>
+      <c r="E243">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="244" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>415637</v>
       </c>
@@ -5215,8 +5593,14 @@
       <c r="C244">
         <v>42481908</v>
       </c>
-    </row>
-    <row r="245" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D244" t="s">
+        <v>475</v>
+      </c>
+      <c r="E244">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="245" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>415638</v>
       </c>
@@ -5226,8 +5610,14 @@
       <c r="C245">
         <v>10357267</v>
       </c>
-    </row>
-    <row r="246" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D245" t="s">
+        <v>476</v>
+      </c>
+      <c r="E245">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="246" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>425825</v>
       </c>
@@ -5237,8 +5627,14 @@
       <c r="C246">
         <v>41081496</v>
       </c>
-    </row>
-    <row r="247" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D246" t="s">
+        <v>481</v>
+      </c>
+      <c r="E246">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="247" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>415663</v>
       </c>
@@ -5248,8 +5644,14 @@
       <c r="C247">
         <v>41872048</v>
       </c>
-    </row>
-    <row r="248" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D247" t="s">
+        <v>485</v>
+      </c>
+      <c r="E247">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="248" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>425853</v>
       </c>
@@ -5259,8 +5661,14 @@
       <c r="C248">
         <v>9668566</v>
       </c>
-    </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D248" t="s">
+        <v>479</v>
+      </c>
+      <c r="E248">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="249" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>425854</v>
       </c>
@@ -5270,8 +5678,14 @@
       <c r="C249">
         <v>42869992</v>
       </c>
-    </row>
-    <row r="250" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D249" t="s">
+        <v>477</v>
+      </c>
+      <c r="E249">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="250" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>425855</v>
       </c>
@@ -5281,8 +5695,14 @@
       <c r="C250">
         <v>48036215</v>
       </c>
-    </row>
-    <row r="251" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D250" t="s">
+        <v>487</v>
+      </c>
+      <c r="E250">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="251" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>425856</v>
       </c>
@@ -5292,8 +5712,14 @@
       <c r="C251">
         <v>44360253</v>
       </c>
-    </row>
-    <row r="252" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D251" t="s">
+        <v>488</v>
+      </c>
+      <c r="E251">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="252" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>426492</v>
       </c>
@@ -5303,8 +5729,14 @@
       <c r="C252">
         <v>47613259</v>
       </c>
-    </row>
-    <row r="253" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D252" t="s">
+        <v>486</v>
+      </c>
+      <c r="E252">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="253" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>425872</v>
       </c>
@@ -5314,8 +5746,14 @@
       <c r="C253">
         <v>9571788</v>
       </c>
-    </row>
-    <row r="254" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D253" t="s">
+        <v>482</v>
+      </c>
+      <c r="E253">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="254" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>415703</v>
       </c>
@@ -5325,8 +5763,14 @@
       <c r="C254">
         <v>42342536</v>
       </c>
-    </row>
-    <row r="255" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D254" t="s">
+        <v>480</v>
+      </c>
+      <c r="E254">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="255" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>415716</v>
       </c>
@@ -5336,8 +5780,14 @@
       <c r="C255">
         <v>9321834</v>
       </c>
-    </row>
-    <row r="256" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D255" t="s">
+        <v>484</v>
+      </c>
+      <c r="E255">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="256" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>425939</v>
       </c>
@@ -5347,8 +5797,14 @@
       <c r="C256">
         <v>47462047</v>
       </c>
-    </row>
-    <row r="257" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D256" t="s">
+        <v>483</v>
+      </c>
+      <c r="E256">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="257" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>415744</v>
       </c>
@@ -5358,8 +5814,14 @@
       <c r="C257">
         <v>40341679</v>
       </c>
-    </row>
-    <row r="258" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D257" t="s">
+        <v>478</v>
+      </c>
+      <c r="E257">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="258" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>426003</v>
       </c>
@@ -5369,8 +5831,14 @@
       <c r="C258">
         <v>46691035</v>
       </c>
-    </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D258" t="s">
+        <v>489</v>
+      </c>
+      <c r="E258">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="259" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>426012</v>
       </c>
@@ -5380,8 +5848,14 @@
       <c r="C259">
         <v>10518811</v>
       </c>
-    </row>
-    <row r="260" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D259" t="s">
+        <v>491</v>
+      </c>
+      <c r="E259">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="260" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>426029</v>
       </c>
@@ -5391,8 +5865,14 @@
       <c r="C260">
         <v>80447049</v>
       </c>
-    </row>
-    <row r="261" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D260" t="s">
+        <v>494</v>
+      </c>
+      <c r="E260">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="261" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>426030</v>
       </c>
@@ -5402,8 +5882,14 @@
       <c r="C261">
         <v>10668721</v>
       </c>
-    </row>
-    <row r="262" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D261" t="s">
+        <v>490</v>
+      </c>
+      <c r="E261">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="262" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>426237</v>
       </c>
@@ -5413,8 +5899,14 @@
       <c r="C262">
         <v>43203309</v>
       </c>
-    </row>
-    <row r="263" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D262" t="s">
+        <v>499</v>
+      </c>
+      <c r="E262">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="263" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>415835</v>
       </c>
@@ -5424,8 +5916,14 @@
       <c r="C263">
         <v>6747711</v>
       </c>
-    </row>
-    <row r="264" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D263" t="s">
+        <v>493</v>
+      </c>
+      <c r="E263">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="264" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>415842</v>
       </c>
@@ -5435,8 +5933,14 @@
       <c r="C264">
         <v>10356600</v>
       </c>
-    </row>
-    <row r="265" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D264" t="s">
+        <v>501</v>
+      </c>
+      <c r="E264">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="265" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>426051</v>
       </c>
@@ -5446,8 +5950,14 @@
       <c r="C265">
         <v>48058641</v>
       </c>
-    </row>
-    <row r="266" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D265" t="s">
+        <v>500</v>
+      </c>
+      <c r="E265">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="266" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>426061</v>
       </c>
@@ -5457,8 +5967,14 @@
       <c r="C266">
         <v>41023917</v>
       </c>
-    </row>
-    <row r="267" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D266" t="s">
+        <v>496</v>
+      </c>
+      <c r="E266">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="267" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A267">
         <v>426590</v>
       </c>
@@ -5468,8 +5984,14 @@
       <c r="C267">
         <v>25765914</v>
       </c>
-    </row>
-    <row r="268" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D267" t="s">
+        <v>492</v>
+      </c>
+      <c r="E267">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="268" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>426766</v>
       </c>
@@ -5479,8 +6001,14 @@
       <c r="C268">
         <v>9043963</v>
       </c>
-    </row>
-    <row r="269" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D268" t="s">
+        <v>495</v>
+      </c>
+      <c r="E268">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="269" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A269">
         <v>426086</v>
       </c>
@@ -5490,8 +6018,14 @@
       <c r="C269">
         <v>41434940</v>
       </c>
-    </row>
-    <row r="270" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D269" t="s">
+        <v>498</v>
+      </c>
+      <c r="E269">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="270" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A270">
         <v>426095</v>
       </c>
@@ -5501,8 +6035,14 @@
       <c r="C270">
         <v>42992960</v>
       </c>
-    </row>
-    <row r="271" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D270" t="s">
+        <v>497</v>
+      </c>
+      <c r="E270">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="271" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>426094</v>
       </c>
@@ -5512,8 +6052,14 @@
       <c r="C271">
         <v>43335784</v>
       </c>
-    </row>
-    <row r="272" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D271" t="s">
+        <v>504</v>
+      </c>
+      <c r="E271">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="272" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A272">
         <v>426142</v>
       </c>
@@ -5523,8 +6069,14 @@
       <c r="C272">
         <v>9218058</v>
       </c>
-    </row>
-    <row r="273" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D272" t="s">
+        <v>502</v>
+      </c>
+      <c r="E272">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="273" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A273">
         <v>426155</v>
       </c>
@@ -5534,8 +6086,14 @@
       <c r="C273">
         <v>46542518</v>
       </c>
-    </row>
-    <row r="274" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D273" t="s">
+        <v>503</v>
+      </c>
+      <c r="E273">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="274" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A274">
         <v>426174</v>
       </c>
@@ -5545,8 +6103,14 @@
       <c r="C274">
         <v>9315832</v>
       </c>
-    </row>
-    <row r="275" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D274" t="s">
+        <v>505</v>
+      </c>
+      <c r="E274">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="275" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>426185</v>
       </c>
@@ -5556,8 +6120,14 @@
       <c r="C275">
         <v>43239978</v>
       </c>
-    </row>
-    <row r="276" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D275" t="s">
+        <v>508</v>
+      </c>
+      <c r="E275">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="276" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A276">
         <v>426187</v>
       </c>
@@ -5567,8 +6137,14 @@
       <c r="C276">
         <v>42781573</v>
       </c>
-    </row>
-    <row r="277" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D276" t="s">
+        <v>507</v>
+      </c>
+      <c r="E276">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="277" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A277">
         <v>415904</v>
       </c>
@@ -5578,8 +6154,14 @@
       <c r="C277">
         <v>44669268</v>
       </c>
-    </row>
-    <row r="278" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D277" t="s">
+        <v>506</v>
+      </c>
+      <c r="E277">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="278" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A278">
         <v>426202</v>
       </c>
@@ -5589,8 +6171,14 @@
       <c r="C278">
         <v>42792032</v>
       </c>
-    </row>
-    <row r="279" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D278" t="s">
+        <v>414</v>
+      </c>
+      <c r="E278">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="279" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A279">
         <v>426215</v>
       </c>
@@ -5600,8 +6188,14 @@
       <c r="C279">
         <v>41740677</v>
       </c>
-    </row>
-    <row r="280" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D279" t="s">
+        <v>413</v>
+      </c>
+      <c r="E279">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="280" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A280">
         <v>426230</v>
       </c>
@@ -5611,8 +6205,14 @@
       <c r="C280">
         <v>21259672</v>
       </c>
-    </row>
-    <row r="281" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D280" t="s">
+        <v>422</v>
+      </c>
+      <c r="E280">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="281" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A281">
         <v>425434</v>
       </c>
@@ -5622,8 +6222,14 @@
       <c r="C281">
         <v>40974095</v>
       </c>
-    </row>
-    <row r="282" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D281" t="s">
+        <v>410</v>
+      </c>
+      <c r="E281">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="282" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A282">
         <v>426308</v>
       </c>
@@ -5633,8 +6239,14 @@
       <c r="C282">
         <v>42812927</v>
       </c>
-    </row>
-    <row r="283" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D282" t="s">
+        <v>389</v>
+      </c>
+      <c r="E282">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="283" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A283">
         <v>426380</v>
       </c>
@@ -5644,8 +6256,14 @@
       <c r="C283">
         <v>46407340</v>
       </c>
-    </row>
-    <row r="284" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D283" t="s">
+        <v>415</v>
+      </c>
+      <c r="E283">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="284" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A284">
         <v>426727</v>
       </c>
@@ -5655,8 +6273,14 @@
       <c r="C284">
         <v>9793589</v>
       </c>
-    </row>
-    <row r="285" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D284" t="s">
+        <v>390</v>
+      </c>
+      <c r="E284">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="285" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A285">
         <v>426280</v>
       </c>
@@ -5666,8 +6290,14 @@
       <c r="C285">
         <v>46599752</v>
       </c>
-    </row>
-    <row r="286" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D285" t="s">
+        <v>387</v>
+      </c>
+      <c r="E285">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="286" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A286">
         <v>425951</v>
       </c>
@@ -5677,8 +6307,14 @@
       <c r="C286">
         <v>80205119</v>
       </c>
-    </row>
-    <row r="287" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D286" t="s">
+        <v>391</v>
+      </c>
+      <c r="E286">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="287" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A287">
         <v>425762</v>
       </c>
@@ -5688,8 +6324,14 @@
       <c r="C287">
         <v>40757255</v>
       </c>
-    </row>
-    <row r="288" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D287" t="s">
+        <v>421</v>
+      </c>
+      <c r="E287">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="288" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A288">
         <v>426100</v>
       </c>
@@ -5699,8 +6341,14 @@
       <c r="C288">
         <v>43587423</v>
       </c>
-    </row>
-    <row r="289" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D288" t="s">
+        <v>392</v>
+      </c>
+      <c r="E288">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="289" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A289">
         <v>426310</v>
       </c>
@@ -5710,8 +6358,14 @@
       <c r="C289">
         <v>41540512</v>
       </c>
-    </row>
-    <row r="290" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D289" t="s">
+        <v>388</v>
+      </c>
+      <c r="E289">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="290" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A290">
         <v>416011</v>
       </c>
@@ -5721,8 +6375,14 @@
       <c r="C290">
         <v>41244558</v>
       </c>
-    </row>
-    <row r="291" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D290" t="s">
+        <v>403</v>
+      </c>
+      <c r="E290">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="291" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A291">
         <v>416021</v>
       </c>
@@ -5732,8 +6392,14 @@
       <c r="C291">
         <v>45379735</v>
       </c>
-    </row>
-    <row r="292" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D291" t="s">
+        <v>401</v>
+      </c>
+      <c r="E291">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="292" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>426366</v>
       </c>
@@ -5743,8 +6409,14 @@
       <c r="C292">
         <v>42293387</v>
       </c>
-    </row>
-    <row r="293" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D292" t="s">
+        <v>400</v>
+      </c>
+      <c r="E292">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="293" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A293">
         <v>426642</v>
       </c>
@@ -5754,8 +6426,14 @@
       <c r="C293">
         <v>41571387</v>
       </c>
-    </row>
-    <row r="294" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D293" t="s">
+        <v>428</v>
+      </c>
+      <c r="E293">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="294" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A294">
         <v>426361</v>
       </c>
@@ -5765,8 +6443,14 @@
       <c r="C294">
         <v>42433753</v>
       </c>
-    </row>
-    <row r="295" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D294" t="s">
+        <v>402</v>
+      </c>
+      <c r="E294">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="295" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A295">
         <v>425608</v>
       </c>
@@ -5776,8 +6460,14 @@
       <c r="C295">
         <v>8339726</v>
       </c>
-    </row>
-    <row r="296" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D295" t="s">
+        <v>420</v>
+      </c>
+      <c r="E295">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="296" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A296">
         <v>426008</v>
       </c>
@@ -5787,8 +6477,14 @@
       <c r="C296">
         <v>44263608</v>
       </c>
-    </row>
-    <row r="297" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D296" t="s">
+        <v>411</v>
+      </c>
+      <c r="E296">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="297" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A297">
         <v>426391</v>
       </c>
@@ -5798,8 +6494,14 @@
       <c r="C297">
         <v>80228446</v>
       </c>
-    </row>
-    <row r="298" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D297" t="s">
+        <v>404</v>
+      </c>
+      <c r="E297">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="298" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A298">
         <v>426006</v>
       </c>
@@ -5809,8 +6511,14 @@
       <c r="C298">
         <v>44537441</v>
       </c>
-    </row>
-    <row r="299" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D298" t="s">
+        <v>407</v>
+      </c>
+      <c r="E298">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="299" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A299">
         <v>426477</v>
       </c>
@@ -5820,8 +6528,14 @@
       <c r="C299">
         <v>25701458</v>
       </c>
-    </row>
-    <row r="300" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D299" t="s">
+        <v>405</v>
+      </c>
+      <c r="E299">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="300" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A300">
         <v>416090</v>
       </c>
@@ -5831,8 +6545,14 @@
       <c r="C300">
         <v>7487696</v>
       </c>
-    </row>
-    <row r="301" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D300" t="s">
+        <v>406</v>
+      </c>
+      <c r="E300">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="301" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A301">
         <v>416097</v>
       </c>
@@ -5842,8 +6562,14 @@
       <c r="C301">
         <v>9218281</v>
       </c>
-    </row>
-    <row r="302" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D301" t="s">
+        <v>408</v>
+      </c>
+      <c r="E301">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="302" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A302">
         <v>426501</v>
       </c>
@@ -5853,8 +6579,14 @@
       <c r="C302">
         <v>10114435</v>
       </c>
-    </row>
-    <row r="303" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D302" t="s">
+        <v>409</v>
+      </c>
+      <c r="E302">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="303" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A303">
         <v>426513</v>
       </c>
@@ -5864,8 +6596,14 @@
       <c r="C303">
         <v>48038919</v>
       </c>
-    </row>
-    <row r="304" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D303" t="s">
+        <v>412</v>
+      </c>
+      <c r="E303">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="304" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A304">
         <v>426519</v>
       </c>

</xml_diff>